<commit_message>
Harm summaries: tools for the weekly run, and the first 3 summaries
- pipeline/scripts/harm_todo.py lists citations still needing a summary, with the
  Care Compare report address
- pipeline/scripts/harm_apply.py writes summaries into harm_summaries.xlsx and adds
  them to the published data.js without a rebuild (never overwrites a summary)
- pipeline/HARM_SUMMARIES.md is the procedure the weekly Claude run follows
- First 3 summaries, from the official reports: Bayberry Commons 12/19/2024 (F0600),
  Saint Elizabeth Home 11/25/2024 (F0805), Lincolnwood 11/25/2024 (F0661)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015nisUc5oGaBRT1cw14rGj4
</commit_message>
<xml_diff>
--- a/pipeline/harm_summaries.xlsx
+++ b/pipeline/harm_summaries.xlsx
@@ -5143,8 +5143,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415080/health/complaint-inspection?date=2024-12-19</t>
         </is>
       </c>
-      <c r="H109" s="4" t="inlineStr"/>
-      <c r="I109" s="3" t="inlineStr"/>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>Staff found a resident with severe dementia on a secured unit in a sexual act with another resident with dementia, who could not consent either. After staff separated them and started 15-minute checks, the two were found in a sexual act again later that evening. The 15-minute checks were not fully done afterward, and no new safety step was added when the other resident's sexual behavior continued two days later.</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -5182,8 +5190,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415010/health/complaint-inspection?date=2024-11-25</t>
         </is>
       </c>
-      <c r="H110" s="4" t="inlineStr"/>
-      <c r="I110" s="3" t="inlineStr"/>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia who was ordered pureed food because of swallowing problems was given regular oatmeal chocolate chip cookies by a nurse, choked, and died despite the Heimlich maneuver. The nurse told surveyors she knew the resident's diet was pureed and that regular cookies were not allowed.</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -5221,8 +5237,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415035/health/complaint-inspection?date=2024-11-25</t>
         </is>
       </c>
-      <c r="H111" s="4" t="inlineStr"/>
-      <c r="I111" s="3" t="inlineStr"/>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>A resident on dialysis was sent home with another resident's medicines in the discharge bag, a cholesterol drug and two blood pressure drugs, and took the other resident's cholesterol drug on two days. The nurse did not check what was in the bag or give the resident or family any medicine instructions.</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Harm citation summaries: batch 1 (18 citations)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PVPrLRkDuJ4YCTTu2Vxqj5
</commit_message>
<xml_diff>
--- a/pipeline/harm_summaries.xlsx
+++ b/pipeline/harm_summaries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Harm citations" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to fill this in" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harm citations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to fill this in" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Harm citations'!$A$1:$I$223</definedName>
@@ -542,8 +542,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415087/health/complaint-inspection?date=2026-08-31</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>A resident was prescribed a blood thinner (Lovenox) based on a weight of 173 that the doctor assumed was in kilograms, though it was in pounds, and received more than twice the proper dose 13 times. The resident had bruising, pain, and swelling of the left arm and was hospitalized on 8/18/2026, where a specialist noted a recent bleed and had the drug held for two weeks.</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -581,8 +589,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415087/health/complaint-inspection?date=2026-08-31</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>The doctor, the nurse practitioner, and several nurses did not stop or question a blood thinner (Lovenox) dose that was more than twice what a resident should have received, even though some of them noticed it was unusually high. The resident got the excessive dose 13 times, then had left arm bruising, pain, and swelling and needed to be hospitalized.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -620,8 +636,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415034/health/complaint-inspection?date=2026-08-18</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia and a history of falls had bed rails installed without the required check for the risk of getting trapped in them. The resident was found dead on the floor beside the bed with the head and neck caught between the bed rail and the mattress, and the medical examiner ruled the death an accident caused by positional asphyxia (not being able to breathe because of body position).</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -5401,8 +5425,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415067/health/health-inspection?date=2024-11-21</t>
         </is>
       </c>
-      <c r="H115" s="4" t="inlineStr"/>
-      <c r="I115" s="3" t="inlineStr"/>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>Three residents who were ordered thickened drinks because of trouble swallowing were served drinks that were not thick enough, because staff used one thickener packet per cup no matter the size and did not measure the drinks. One of them, who had recently returned from the hospital after pneumonia, said they choke and cough on the drinks, and inspectors found residents were in immediate jeopardy.</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
@@ -5440,8 +5472,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415067/health/health-inspection?date=2024-11-21</t>
         </is>
       </c>
-      <c r="H116" s="4" t="inlineStr"/>
-      <c r="I116" s="3" t="inlineStr"/>
+      <c r="H116" s="4" t="inlineStr">
+        <is>
+          <t>A resident's suprapubic catheter (a tube through the belly into the bladder) was not changed for about 20 weeks because staff never got an order to change it, and a missed urology appointment was never rescheduled. The resident had severe pain, blood in the urine, leaking, and a suspected urinary tract infection, and was sent to the hospital twice in October 2024.</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -5479,8 +5519,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415079/health/complaint-inspection?date=2024-11-20</t>
         </is>
       </c>
-      <c r="H117" s="4" t="inlineStr"/>
-      <c r="I117" s="3" t="inlineStr"/>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia on a locked unit, who had tried to get on the elevator twice the day before, was not given a wander alarm bracelet or frequent checks as the facility's policy required. The resident left the building without staff noticing and was found by a jogger about 1.5 miles away, and the facility only learned of it when the hospital called.</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
@@ -5518,8 +5566,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415071/health/complaint-inspection?date=2024-11-18</t>
         </is>
       </c>
-      <c r="H118" s="4" t="inlineStr"/>
-      <c r="I118" s="3" t="inlineStr"/>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe dementia had a bed pushed against the wall next to an electric baseboard heater, and staff found the resident's left foot resting directly on the heater. The resident had second-degree burns to the heel, the sole, and the bunion area and was admitted to a hospital intensive care unit. Heaters in the building measured 163 to 190 degrees Fahrenheit, and other residents' beds were also against them.</t>
+        </is>
+      </c>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -5557,8 +5613,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415091/health/health-inspection?date=2024-11-04</t>
         </is>
       </c>
-      <c r="H119" s="4" t="inlineStr"/>
-      <c r="I119" s="3" t="inlineStr"/>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>Three residents ordered a ground diet because of trouble chewing or swallowing were served foods like whole toast, garlic bread, whole grilled cheese sandwiches, dry rolls, and watermelon with seeds, and several staff serving them did not know their diet orders. One resident was seen coughing while eating, and inspectors found residents were in immediate jeopardy.</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
@@ -5596,8 +5660,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415031/health/health-inspection?date=2024-10-31</t>
         </is>
       </c>
-      <c r="H120" s="4" t="inlineStr"/>
-      <c r="I120" s="3" t="inlineStr"/>
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>Three residents with ostomies (an opening in the belly where stool drains into a bag) had no orders for when to change the bag or what size to use, and the bags were changed when they leaked or came loose. One resident's skin around the opening broke down, burned, and bled with no treatment and no doctor notified, and another resident had a prolapsed stoma with a treatment order the doctor did not know about and staff did not record giving.</t>
+        </is>
+      </c>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -5635,8 +5707,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415050/health/complaint-inspection?date=2024-10-31</t>
         </is>
       </c>
-      <c r="H121" s="4" t="inlineStr"/>
-      <c r="I121" s="3" t="inlineStr"/>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>When a resident with heart failure and an irregular heart rhythm came back from the hospital, staff entered medication orders from a list of medicines taken before the hospital stay instead of the hospital's discharge orders. The resident went 16 days without a prescribed heart rhythm drug (amiodarone), an inhaler, and a water pill, and was sent back to the hospital with trouble breathing and a fast, irregular heartbeat.</t>
+        </is>
+      </c>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -5674,8 +5754,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415038/health/complaint-inspection?date=2024-10-21</t>
         </is>
       </c>
-      <c r="H122" s="4" t="inlineStr"/>
-      <c r="I122" s="3" t="inlineStr"/>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia who was known to wander into other rooms and strike out hit another resident on the head and face with a commode cover, and a hospital scan showed a broken upper jaw bone. In a separate incident, a different resident with dementia punched a resident who had tried to get them to leave their room, causing a bloody lip.</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -5713,8 +5801,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415035/health/complaint-inspection?date=2024-10-17</t>
         </is>
       </c>
-      <c r="H123" s="4" t="inlineStr"/>
-      <c r="I123" s="3" t="inlineStr"/>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia whose care plan called for two staff to turn in bed was turned by one nursing assistant alone, who then turned away to get wipes. The resident rolled off the bed, hit their face on a chair, and landed on the floor, with cuts to the forehead and the back of the head that needed emergency room care and stitches.</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
@@ -5752,8 +5848,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415129/health/complaint-inspection?date=2024-10-15</t>
         </is>
       </c>
-      <c r="H124" s="4" t="inlineStr"/>
-      <c r="I124" s="3" t="inlineStr"/>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>A resident with memory problems walked out of the building with a walker at 2:41 PM, and staff did not notice the resident was missing until about 8:45 PM and did not call police until 11:05 PM. The resident got lost and was found by police at a coffee shop in Woonsocket, about 13 miles away, and taken to a hospital around 4 AM. When the resident came back, the facility added no safety measures such as checks or a wander alarm.</t>
+        </is>
+      </c>
+      <c r="I124" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -5791,8 +5895,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415108/health/health-inspection?date=2024-10-11</t>
         </is>
       </c>
-      <c r="H125" s="4" t="inlineStr"/>
-      <c r="I125" s="3" t="inlineStr"/>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>A resident at risk for pressure sores had no weekly skin checks for 8 weeks and no treatment for a heel that the director of nursing noticed was mushy soon after admission. The heel turned black and became a deep wound with dead tissue that had to be surgically removed, and a new treatment the wound doctor recommended was not started for 8 days.</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -5830,8 +5942,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415110/health/complaint-inspection?date=2024-10-08</t>
         </is>
       </c>
-      <c r="H126" s="4" t="inlineStr"/>
-      <c r="I126" s="3" t="inlineStr"/>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>A nurse prepared medicines for two residents at the same time and gave one resident a strong antipsychotic drug (Clozaril, 125 mg) meant for the other. The resident became unresponsive with low oxygen, was admitted to a hospital critical care unit, needed a breathing tube, and was treated for an abnormal heart rhythm reading.</t>
+        </is>
+      </c>
+      <c r="I126" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -5869,8 +5989,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415027/health/complaint-inspection?date=2024-10-02</t>
         </is>
       </c>
-      <c r="H127" s="4" t="inlineStr"/>
-      <c r="I127" s="3" t="inlineStr"/>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>A resident being treated with an antibiotic for a blood infection missed four doses in a row because a nurse entered the wrong start date and the liquid form had not arrived, even though tablets were on hand, and no provider was told. Three days after arriving, the resident had a fever of 103.9, a racing heart, and severe belly pain and was sent to the hospital with urosepsis (a serious infection that spread from the urinary tract).</t>
+        </is>
+      </c>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
@@ -5908,8 +6036,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415110/health/complaint-inspection?date=2024-10-01</t>
         </is>
       </c>
-      <c r="H128" s="4" t="inlineStr"/>
-      <c r="I128" s="3" t="inlineStr"/>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>A resident tearfully told staff on a Sunday that another resident was moving too fast and trying to get into bed with them, but staff only suggested talking to social services the next day and took no steps to keep the resident safe. The resident reported being sexually assaulted that night and was treated at a hospital for pelvic and genital pain.</t>
+        </is>
+      </c>
+      <c r="I128" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -5947,8 +6083,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415110/health/complaint-inspection?date=2024-10-01</t>
         </is>
       </c>
-      <c r="H129" s="4" t="inlineStr"/>
-      <c r="I129" s="3" t="inlineStr"/>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>Several staff heard a resident's worries about another resident but did not recognize them as possible abuse, look into them, or protect the resident. After the resident reported being sexually assaulted and was treated at a hospital, the facility could not show that it had started an investigation or kept the resident safe from further abuse.</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Harm citation summaries: batch 2 (23 citations)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PVPrLRkDuJ4YCTTu2Vxqj5
</commit_message>
<xml_diff>
--- a/pipeline/harm_summaries.xlsx
+++ b/pipeline/harm_summaries.xlsx
@@ -6130,8 +6130,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/complaint-inspection?date=2024-09-25</t>
         </is>
       </c>
-      <c r="H130" s="4" t="inlineStr"/>
-      <c r="I130" s="3" t="inlineStr"/>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t>When a resident with a seizure disorder came back from the hospital, the admission was never finished, so no medication orders were entered and the resident got none of their medicines, including seizure drugs, from 3 PM one day until about 1:45 PM the next. The resident then had two seizures and was sent back to the hospital, where they were admitted with seizures and respiratory failure.</t>
+        </is>
+      </c>
+      <c r="I130" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -6169,8 +6177,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/complaint-inspection?date=2024-09-12</t>
         </is>
       </c>
-      <c r="H131" s="4" t="inlineStr"/>
-      <c r="I131" s="3" t="inlineStr"/>
+      <c r="H131" s="4" t="inlineStr">
+        <is>
+          <t>Staff found a resident with dementia and depression with a belt wrapped around their neck in the middle of the night, but did not put the resident on constant one-to-one watch, did not tell the doctor, nursing leaders, or family, and left belts and cords in the room. Later that day the resident walked out of the building alone twice, and was seen wearing a belt, before being sent to the hospital for a psychiatric evaluation.</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
@@ -6208,8 +6224,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/complaint-inspection?date=2024-09-12</t>
         </is>
       </c>
-      <c r="H132" s="4" t="inlineStr"/>
-      <c r="I132" s="3" t="inlineStr"/>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>After a resident tried to hang themselves with a belt during the night, staff did not provide the one-to-one supervision the facility's policy required, kept no record of safety checks, and left belts, string ties, and cords in the room. The resident left the unit and the building unsupervised twice that same day before being sent to the hospital.</t>
+        </is>
+      </c>
+      <c r="I132" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -6247,8 +6271,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415033/health/health-inspection?date=2024-09-06</t>
         </is>
       </c>
-      <c r="H133" s="4" t="inlineStr"/>
-      <c r="I133" s="3" t="inlineStr"/>
+      <c r="H133" s="4" t="inlineStr">
+        <is>
+          <t>The kitchen dishwasher was not sanitizing dishes, because the sanitizer was below the required level and staff had no correct test strips to check it, which put residents at risk of foodborne illness. Inspectors also found egg, ham, and seafood salad sandwiches held at about 49 to 50 degrees, meat thawing at room temperature, a dirty ice machine chute, and built-up grease and grime.</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
@@ -6286,8 +6318,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415033/health/health-inspection?date=2024-09-06</t>
         </is>
       </c>
-      <c r="H134" s="4" t="inlineStr"/>
-      <c r="I134" s="3" t="inlineStr"/>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>A resident's heel pressure wound, which had healed in late August, reopened, but it had no dressing or treatment order, a weekly skin check was missed, and the doctor was not told until an inspector found it. A nurse had put a skin protectant on it that should not be used on open wounds, and the resident said the heel hurt at times.</t>
+        </is>
+      </c>
+      <c r="I134" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -6325,8 +6365,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415035/health/complaint-inspection?date=2024-08-29</t>
         </is>
       </c>
-      <c r="H135" s="4" t="inlineStr"/>
-      <c r="I135" s="3" t="inlineStr"/>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>A nurse gave a resident their roommate's medicines, including two blood pressure drugs, without checking that they were for the right person. The resident's blood pressure dropped too low and the resident needed IV fluids.</t>
+        </is>
+      </c>
+      <c r="I135" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
@@ -6364,8 +6412,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415063/health/health-inspection?date=2024-08-22</t>
         </is>
       </c>
-      <c r="H136" s="4" t="inlineStr"/>
-      <c r="I136" s="3" t="inlineStr"/>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>During a COVID-19 outbreak, staff cleaned shared blood pressure cuffs and stethoscopes with wipes that do not kill the COVID-19 virus, and several staff went into rooms of residents with COVID-19 without the required N95 mask or eye protection. A nurse also skipped the required gown for a resident with MRSA (a drug-resistant infection), and a resident with a urinary catheter was not on required precautions, putting many residents at risk of infection.</t>
+        </is>
+      </c>
+      <c r="I136" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -6403,8 +6459,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415063/health/health-inspection?date=2024-08-22</t>
         </is>
       </c>
-      <c r="H137" s="4" t="inlineStr"/>
-      <c r="I137" s="3" t="inlineStr"/>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>A resident who had impulse control problems after a stroke yelled at a resident with severe dementia and hit them about three times on the arm, which a staff witness said was unprovoked. The resident with dementia had two skin tears.</t>
+        </is>
+      </c>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
@@ -6442,8 +6506,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415063/health/health-inspection?date=2024-08-22</t>
         </is>
       </c>
-      <c r="H138" s="4" t="inlineStr"/>
-      <c r="I138" s="3" t="inlineStr"/>
+      <c r="H138" s="4" t="inlineStr">
+        <is>
+          <t>A resident with schizophrenia missed a scheduled antipsychotic injection because staff never entered the rescheduled order. The resident's psychosis returned, with hearing voices and saying they wanted to stab people, and the resident needed extra medicine and safety checks every 15 minutes.</t>
+        </is>
+      </c>
+      <c r="I138" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -6481,8 +6553,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415075/health/complaint-inspection?date=2024-08-22</t>
         </is>
       </c>
-      <c r="H139" s="4" t="inlineStr"/>
-      <c r="I139" s="3" t="inlineStr"/>
+      <c r="H139" s="4" t="inlineStr">
+        <is>
+          <t>A resident with poor blood flow to the legs had wounds between the toes that a nurse's skin check missed because she did not look between the toes. The next day the resident went to the hospital, where staff found black tissue and maggots in the wounds and admitted the resident with a skin infection treated with IV antibiotics.</t>
+        </is>
+      </c>
+      <c r="I139" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
@@ -6520,8 +6600,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415075/health/complaint-inspection?date=2024-08-22</t>
         </is>
       </c>
-      <c r="H140" s="4" t="inlineStr"/>
-      <c r="I140" s="3" t="inlineStr"/>
+      <c r="H140" s="4" t="inlineStr">
+        <is>
+          <t>The facility had not trained or tested its nurses on how to do skin checks. A nurse's skin check missed wounds between a resident's toes, and the next day hospital staff found black tissue and maggots in the wounds and admitted the resident with a skin infection.</t>
+        </is>
+      </c>
+      <c r="I140" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -6559,8 +6647,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/complaint-inspection?date=2024-08-22</t>
         </is>
       </c>
-      <c r="H141" s="4" t="inlineStr"/>
-      <c r="I141" s="3" t="inlineStr"/>
+      <c r="H141" s="4" t="inlineStr">
+        <is>
+          <t>Residents with dementia who were known to be at risk of wandering away in their wheelchairs were not supervised. One resident left and was found at a convenience store about 0.2 miles away. Another had earlier reached the same store by a route with no sidewalks that means wheeling onto busy Route 3, and during the inspection was found down the street and then outside alone again.</t>
+        </is>
+      </c>
+      <c r="I141" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
@@ -6598,8 +6694,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415064/health/complaint-inspection?date=2024-08-16</t>
         </is>
       </c>
-      <c r="H142" s="4" t="inlineStr"/>
-      <c r="I142" s="3" t="inlineStr"/>
+      <c r="H142" s="4" t="inlineStr">
+        <is>
+          <t>The administrator ordered the housekeeping director, who had tested positive for COVID-19, to work as the only cook for all residents for two days, even though she did not have the required food safety manager certification. Afterward 26 residents tested positive for COVID-19, though none had been positive before she worked.</t>
+        </is>
+      </c>
+      <c r="I142" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -6637,8 +6741,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415064/health/complaint-inspection?date=2024-08-16</t>
         </is>
       </c>
-      <c r="H143" s="4" t="inlineStr"/>
-      <c r="I143" s="3" t="inlineStr"/>
+      <c r="H143" s="4" t="inlineStr">
+        <is>
+          <t>A staff member who had tested positive for COVID-19 was allowed to work as the cook during her isolation period, preparing meals over two days without a mask. Within days, 26 residents tested positive for COVID-19, where no residents had been positive before.</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
@@ -6676,8 +6788,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415031/health/complaint-inspection?date=2024-08-13</t>
         </is>
       </c>
-      <c r="H144" s="4" t="inlineStr"/>
-      <c r="I144" s="3" t="inlineStr"/>
+      <c r="H144" s="4" t="inlineStr">
+        <is>
+          <t>A resident told staff their roommate, who has dementia, had put a blanket over their face and seemed to be trying to kill them. Staff moved that resident out but moved in a resident on hospice who had severe dementia, could not walk, and depended on staff for all care. The next night staff heard screaming and found the roommate on top of the hospice resident, holding a sheet over the resident's face.</t>
+        </is>
+      </c>
+      <c r="I144" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -6715,8 +6835,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415031/health/complaint-inspection?date=2024-08-13</t>
         </is>
       </c>
-      <c r="H145" s="4" t="inlineStr"/>
-      <c r="I145" s="3" t="inlineStr"/>
+      <c r="H145" s="4" t="inlineStr">
+        <is>
+          <t>When a resident reported that their roommate had put a blanket over their face and seemed to be trying to kill them, staff moved the resident but did not investigate, saying they were too busy. A resident on hospice with severe dementia was moved into that room the same day, and the next night the roommate was found on top of the hospice resident, holding a sheet over the resident's face.</t>
+        </is>
+      </c>
+      <c r="I145" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
@@ -6754,8 +6882,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415074/health/complaint-inspection?date=2024-08-06</t>
         </is>
       </c>
-      <c r="H146" s="4" t="inlineStr"/>
-      <c r="I146" s="3" t="inlineStr"/>
+      <c r="H146" s="4" t="inlineStr">
+        <is>
+          <t>A resident with Alzheimer's disease who needed two staff to move in bed was found wedged between the bed and the wall, and one nursing assistant moved the resident back alone. Days later the resident had new bruises and left leg and hip pain, an X-ray showed a broken left thigh bone near the hip, and the resident needed regular morphine for pain.</t>
+        </is>
+      </c>
+      <c r="I146" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -6793,8 +6929,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415080/health/complaint-inspection?date=2024-08-05</t>
         </is>
       </c>
-      <c r="H147" s="4" t="inlineStr"/>
-      <c r="I147" s="3" t="inlineStr"/>
+      <c r="H147" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe memory problems who was at high risk for falls was supposed to wear hip protectors, but was not wearing them when they tripped while walking with a nursing assistant. The resident fell on the right hip and was taken to the hospital with a broken hip.</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
@@ -6832,8 +6976,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415031/health/complaint-inspection?date=2024-08-02</t>
         </is>
       </c>
-      <c r="H148" s="4" t="inlineStr"/>
-      <c r="I148" s="3" t="inlineStr"/>
+      <c r="H148" s="4" t="inlineStr">
+        <is>
+          <t>A resident with no teeth who was on a minced and moist diet and needed supervision while eating was given two whole slices of pizza by another resident. A nurse knew about it but left the resident alone twice while they ate it. The resident choked, could not be revived despite the Heimlich maneuver and CPR, and died at the hospital.</t>
+        </is>
+      </c>
+      <c r="I148" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -6871,8 +7023,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415091/health/complaint-inspection?date=2024-07-30</t>
         </is>
       </c>
-      <c r="H149" s="4" t="inlineStr"/>
-      <c r="I149" s="3" t="inlineStr"/>
+      <c r="H149" s="4" t="inlineStr">
+        <is>
+          <t>A resident deliberately hit their roommate in the leg with a trash can. The roommate had an open wound on the shin that needed dressing changes for about a month and left a visible scar.</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
@@ -6910,8 +7070,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415091/health/complaint-inspection?date=2024-07-30</t>
         </is>
       </c>
-      <c r="H150" s="4" t="inlineStr"/>
-      <c r="I150" s="3" t="inlineStr"/>
+      <c r="H150" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe memory problems who uses a wheelchair left the unit, took the elevator, and went out the front door with no staff watching. The wheelchair rolled down the parking lot and the resident fell out where the lot meets the street, with a bleeding bump on the forehead, facial bruising, and skin tears, and was taken to the hospital.</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -6949,8 +7117,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415049/health/complaint-inspection?date=2024-07-17</t>
         </is>
       </c>
-      <c r="H151" s="4" t="inlineStr"/>
-      <c r="I151" s="3" t="inlineStr"/>
+      <c r="H151" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia and a brain injury who had been assessed as a moderate wandering risk had no measures in place to prevent it, and was last seen sitting outside near the front door. A member of the public found the resident lying in a road about 1 mile away, wearing heavy clothing and sweating heavily, and the resident was taken to the hospital unsure of where they were.</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
@@ -6988,8 +7164,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415035/health/complaint-inspection?date=2024-06-27</t>
         </is>
       </c>
-      <c r="H152" s="4" t="inlineStr"/>
-      <c r="I152" s="3" t="inlineStr"/>
+      <c r="H152" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia and a history of aggression went into another resident's room and went through their belongings, and the resident living there said they were pushed when they asked the intruder to leave. The resident who fell was found bleeding from the back of the head with a broken hip, declined surgery, was treated with morphine for pain, and later died.</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Harm citation summaries: batch 3 (19 citations)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PVPrLRkDuJ4YCTTu2Vxqj5
</commit_message>
<xml_diff>
--- a/pipeline/harm_summaries.xlsx
+++ b/pipeline/harm_summaries.xlsx
@@ -7211,8 +7211,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415049/health/complaint-inspection?date=2024-06-24</t>
         </is>
       </c>
-      <c r="H153" s="4" t="inlineStr"/>
-      <c r="I153" s="3" t="inlineStr"/>
+      <c r="H153" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe dementia on a locked unit was sexually abused by another resident with severe dementia, who was found on the resident's bed stroking their genitals. Earlier that night staff had left the other resident alone in the room for over an hour when they could not get them to leave, and staff had not acted on that resident's earlier sexual and intimidating behavior.</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
@@ -7250,8 +7258,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415110/health/complaint-inspection?date=2024-06-24</t>
         </is>
       </c>
-      <c r="H154" s="4" t="inlineStr"/>
-      <c r="I154" s="3" t="inlineStr"/>
+      <c r="H154" s="4" t="inlineStr">
+        <is>
+          <t>A resident recovering from hip surgery, with a history of blood clots, had growing swelling in the left leg, but staff did not check for signs of a clot and no ultrasound was ordered for 5 days, until the surgeon called for one. The ultrasound found blood clots blocking four major veins in the leg, and the resident was hospitalized for IV blood thinners and a procedure to remove the clots.</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
@@ -7289,8 +7305,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415002/health/health-inspection?date=2024-06-17</t>
         </is>
       </c>
-      <c r="H155" s="4" t="inlineStr"/>
-      <c r="I155" s="3" t="inlineStr"/>
+      <c r="H155" s="4" t="inlineStr">
+        <is>
+          <t>A resident with swallowing problems who had been hospitalized for inhaling food was ordered one-on-one help at every meal and thickened drinks, but was seen eating alone, drinking unthickened coffee, and coughing, and staff and the doctor did not know about the order. Another resident with severe dementia was left alone with foods like whole sausage, clam cakes, and bacon instead of the soft, bite-sized food ordered, and was seen struggling to chew and coughing.</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
@@ -7328,8 +7352,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/complaint-inspection?date=2024-06-13</t>
         </is>
       </c>
-      <c r="H156" s="4" t="inlineStr"/>
-      <c r="I156" s="3" t="inlineStr"/>
+      <c r="H156" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe dementia, who staff had brought back from the front doors the day before, got out of the building alone in a wheelchair and was found struggling to move in a lane of a busy main road while cars went around them. The resident wore only slipper socks, the oxygen tube was on their forehead, and staff did not know the resident was gone until a worker from a nearby facility brought them back.</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -7367,8 +7399,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/complaint-inspection?date=2024-06-06</t>
         </is>
       </c>
-      <c r="H157" s="4" t="inlineStr"/>
-      <c r="I157" s="3" t="inlineStr"/>
+      <c r="H157" s="4" t="inlineStr">
+        <is>
+          <t>A resident with a tracheostomy (a breathing tube in the neck) who can communicate only by blinking and using a letter board said a nurse forced mouthwash into their mouth without suctioning, and they swallowed it. The nurse had never worked with these residents and had not been trained, and the facility had no procedure for safe mouth care for the 15 residents with tracheostomies, which inspectors found put them in immediate jeopardy.</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
@@ -7406,8 +7446,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415049/health/complaint-inspection?date=2024-06-04</t>
         </is>
       </c>
-      <c r="H158" s="4" t="inlineStr"/>
-      <c r="I158" s="3" t="inlineStr"/>
+      <c r="H158" s="4" t="inlineStr">
+        <is>
+          <t>A resident with cancer had severe, worsening leg swelling, new leg wounds, and a fall that were not reported to a provider or treated, and a daily belly measurement was skipped because there was no tape measure. The resident went to the hospital with severe leg pain, was found to have a blood clot in the right leg, and had 4,800 milliliters of fluid drained from the belly. Staff also did not tell a provider when another resident twice became unresponsive.</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -7445,8 +7493,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/complaint-inspection?date=2024-05-23</t>
         </is>
       </c>
-      <c r="H159" s="4" t="inlineStr"/>
-      <c r="I159" s="3" t="inlineStr"/>
+      <c r="H159" s="4" t="inlineStr">
+        <is>
+          <t>A resident with poor circulation developed purple, cold toes and feet, but an urgent ultrasound was ordered for the wrong foot, the artery scan was never done, and nurses did not tell the provider as the feet got worse. The resident was sent to the hospital two days after the first order with discolored, cold feet and a racing heart, and was started on a blood thinner drip and antibiotics for a leg skin infection with bacteria in the blood.</t>
+        </is>
+      </c>
+      <c r="I159" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
@@ -7484,8 +7540,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415120/health/health-inspection?date=2024-05-23</t>
         </is>
       </c>
-      <c r="H160" s="4" t="inlineStr"/>
-      <c r="I160" s="3" t="inlineStr"/>
+      <c r="H160" s="4" t="inlineStr">
+        <is>
+          <t>Staff did not reweigh residents after big weight changes or take monthly weights as required for 7 residents. One resident fed through a stomach tube lost about 26 pounds, about 14 percent of their body weight, in about a month, and no new steps were added to prevent more weight loss.</t>
+        </is>
+      </c>
+      <c r="I160" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -7523,8 +7587,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/complaint-inspection?date=2024-05-14</t>
         </is>
       </c>
-      <c r="H161" s="4" t="inlineStr"/>
-      <c r="I161" s="3" t="inlineStr"/>
+      <c r="H161" s="4" t="inlineStr">
+        <is>
+          <t>A person without a nursing license was scheduled as the only nurse, with no supervision, for a unit of 34 residents on an overnight shift, and recorded giving medicines including morphine, tube feedings, and breathing treatments. A registered nurse at the facility also worked 20 hours in a 24-hour period.</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
@@ -7562,8 +7634,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/complaint-inspection?date=2024-05-14</t>
         </is>
       </c>
-      <c r="H162" s="4" t="inlineStr"/>
-      <c r="I162" s="3" t="inlineStr"/>
+      <c r="H162" s="4" t="inlineStr">
+        <is>
+          <t>Facility leaders let a person without a nursing license work unsupervised as the nurse for 34 residents on an overnight shift, giving medicines and treatments and doing assessments. The facility had no record of her license, nursing training, or skills checks.</t>
+        </is>
+      </c>
+      <c r="I162" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -7601,8 +7681,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415039/health/complaint-inspection?date=2024-05-09</t>
         </is>
       </c>
-      <c r="H163" s="4" t="inlineStr"/>
-      <c r="I163" s="3" t="inlineStr"/>
+      <c r="H163" s="4" t="inlineStr">
+        <is>
+          <t>A resident with memory problems who was a known risk for leaving, and had left before, was dropped off alone at an outside appointment after staff removed the resident's wander alarm bracelet. The resident took several buses and was found hours later by a facility social worker, standing at the corner of a busy main road about 8 miles away.</t>
+        </is>
+      </c>
+      <c r="I163" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
@@ -7640,8 +7728,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415082/health/complaint-inspection?date=2024-05-08</t>
         </is>
       </c>
-      <c r="H164" s="4" t="inlineStr"/>
-      <c r="I164" s="3" t="inlineStr"/>
+      <c r="H164" s="4" t="inlineStr">
+        <is>
+          <t>Staff made repeated mistakes entering orders for the blood thinner Coumadin for 7 residents, which caused missed doses and wrong doses, including one resident who got the wrong dose for 14 days. Another resident was given Coumadin after a provider ordered it held for a high blood test result, then fell and was found at the hospital to have a dangerously high clotting level (INR of 10.7) that needed medicine to bring it down.</t>
+        </is>
+      </c>
+      <c r="I164" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -7679,8 +7775,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415087/health/complaint-inspection?date=2024-05-08</t>
         </is>
       </c>
-      <c r="H165" s="4" t="inlineStr"/>
-      <c r="I165" s="3" t="inlineStr"/>
+      <c r="H165" s="4" t="inlineStr">
+        <is>
+          <t>Staff regularly boxed in two residents with severe dementia who were at risk of falling, using a wall, a table, a chair, and another resident's recliner so they could not get up, with no assessment, consent, or doctor's order. One resident was pinned in a wheelchair with a table pushed against their chest, and a nurse had allowed the practice.</t>
+        </is>
+      </c>
+      <c r="I165" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
@@ -7718,8 +7822,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415087/health/complaint-inspection?date=2024-05-08</t>
         </is>
       </c>
-      <c r="H166" s="4" t="inlineStr"/>
-      <c r="I166" s="3" t="inlineStr"/>
+      <c r="H166" s="4" t="inlineStr">
+        <is>
+          <t>Two nursing assistants told the nurse in charge they heard a resident with dementia screaming "don't hit me, stop hitting me" while two staff members were in the room, but the nurse did not report or act on it, and the two staff kept working. About 5 hours later, those same two staff members were recorded on video shoving and restraining another resident.</t>
+        </is>
+      </c>
+      <c r="I166" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -7757,8 +7869,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415087/health/complaint-inspection?date=2024-05-08</t>
         </is>
       </c>
-      <c r="H167" s="4" t="inlineStr"/>
-      <c r="I167" s="3" t="inlineStr"/>
+      <c r="H167" s="4" t="inlineStr">
+        <is>
+          <t>Video showed a nursing assistant forcefully shove a resident with severe dementia who was trying to get out of a recliner and yank the resident's legs down. Minutes later she held the resident's arms up while a medication technician pushed a table against the resident's chest, wedging the resident in place, and the resident had scattered bruising on both arms.</t>
+        </is>
+      </c>
+      <c r="I167" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
@@ -7796,8 +7916,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/health-inspection?date=2024-05-08</t>
         </is>
       </c>
-      <c r="H168" s="4" t="inlineStr"/>
-      <c r="I168" s="3" t="inlineStr"/>
+      <c r="H168" s="4" t="inlineStr">
+        <is>
+          <t>Four residents with swallowing problems who were ordered thickened drinks were given drinks that were too thin, and staff and the director of nursing did not know how to make the pudding-thick drinks some of them needed. One of these residents was being treated for pneumonia from inhaling food or liquid and needed suctioning, and another was served thin drinks with straws.</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -7835,8 +7963,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/health-inspection?date=2024-05-08</t>
         </is>
       </c>
-      <c r="H169" s="4" t="inlineStr"/>
-      <c r="I169" s="3" t="inlineStr"/>
+      <c r="H169" s="4" t="inlineStr">
+        <is>
+          <t>Staff did not follow the facility's steps for treating constipation for two residents. One went 5 days without a bowel movement, became very ill with pain and vomiting, and had a stalled bowel (ileus) at the time of their death, and the other went 12 days. A nurse also did not follow a resident's wound care orders and left one of three leg wounds without a dressing.</t>
+        </is>
+      </c>
+      <c r="I169" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
@@ -7874,8 +8010,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/complaint-inspection?date=2024-04-23</t>
         </is>
       </c>
-      <c r="H170" s="4" t="inlineStr"/>
-      <c r="I170" s="3" t="inlineStr"/>
+      <c r="H170" s="4" t="inlineStr">
+        <is>
+          <t>A resident with schizoaffective disorder, a brain injury, and an intellectual disability ran out of an outside appointment and was missing for about 6 hours, but the facility did not assess the resident's risk of leaving or add any safety measures. Two months later the resident left the building twice in two days and was picked up by police and taken to the hospital, confused and in distress.</t>
+        </is>
+      </c>
+      <c r="I170" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -7913,8 +8057,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/health-inspection?date=2024-04-08</t>
         </is>
       </c>
-      <c r="H171" s="4" t="inlineStr"/>
-      <c r="I171" s="3" t="inlineStr"/>
+      <c r="H171" s="4" t="inlineStr">
+        <is>
+          <t>A resident who cannot speak and gets all food, fluids, and medicine through a stomach tube went about 36 hours without any of them after the tube came out, because staff did not follow up on an unclear X-ray meant to confirm the new tube's position. The resident was grimacing in pain, and staff did not tell the family or the provider that the tube had come out.</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Harm citation summaries: batch 4 (23 citations)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PVPrLRkDuJ4YCTTu2Vxqj5
</commit_message>
<xml_diff>
--- a/pipeline/harm_summaries.xlsx
+++ b/pipeline/harm_summaries.xlsx
@@ -8104,8 +8104,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/complaint-inspection?date=2024-04-04</t>
         </is>
       </c>
-      <c r="H172" s="4" t="inlineStr"/>
-      <c r="I172" s="3" t="inlineStr"/>
+      <c r="H172" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe memory problems who often tried to leave and kept taking off their wander alarm bracelet got outside twice in March without it. The first time the resident was found lying on the ground with a finger wound, and no new safety steps followed. The second time, a passerby saw the resident fall twice near the street and helped them back to the door, with no staff in sight.</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -8143,8 +8151,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415023/health/health-inspection?date=2024-03-25</t>
         </is>
       </c>
-      <c r="H173" s="4" t="inlineStr"/>
-      <c r="I173" s="3" t="inlineStr"/>
+      <c r="H173" s="4" t="inlineStr">
+        <is>
+          <t>A resident with dementia vomited several times over two shifts and looked pale and tired, but nurses did not do a full check with vital signs or tell a doctor. The next morning the resident was found unresponsive with no pulse and died after attempts to restart the heart.</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
@@ -8182,8 +8198,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415008/health/health-inspection?date=2024-03-22</t>
         </is>
       </c>
-      <c r="H174" s="4" t="inlineStr"/>
-      <c r="I174" s="3" t="inlineStr"/>
+      <c r="H174" s="4" t="inlineStr">
+        <is>
+          <t>Hot water in residents' rooms, showers, and tubs on 5 of 6 units measured as high as 135 degrees Fahrenheit, well above the state limit of 118 degrees, and staff tested it by hand instead of with a thermometer. Residents who wash on their own said the water gets very hot, and one said they felt they could burn their hands.</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -8221,8 +8245,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415008/health/health-inspection?date=2024-03-22</t>
         </is>
       </c>
-      <c r="H175" s="4" t="inlineStr"/>
-      <c r="I175" s="3" t="inlineStr"/>
+      <c r="H175" s="4" t="inlineStr">
+        <is>
+          <t>A resident who needed two staff to turn in bed asked early in the morning to be repositioned because of pain in the buttocks, but was told to wait for the next shift, and the nursing assistant did not tell the nurse. A few hours later a new open pressure sore was found on the buttocks, and the resident rated the pain 8 out of 10.</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
@@ -8260,8 +8292,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415079/health/health-inspection?date=2024-03-15</t>
         </is>
       </c>
-      <c r="H176" s="4" t="inlineStr"/>
-      <c r="I176" s="3" t="inlineStr"/>
+      <c r="H176" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe dementia and a deep pressure wound was left in a recliner with no pressure-relieving cushion for about 4 hours, soaked in loose stool that had also soaked the wound dressing. New pressure injuries were found on the right hip, the left thigh, and the right buttock, and a nurse had treated one without telling the doctor or getting an order.</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -8299,8 +8339,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415079/health/health-inspection?date=2024-03-15</t>
         </is>
       </c>
-      <c r="H177" s="4" t="inlineStr"/>
-      <c r="I177" s="3" t="inlineStr"/>
+      <c r="H177" s="4" t="inlineStr">
+        <is>
+          <t>A resident who was losing weight and had a poor appetite never got the supplement and appetite medicine the dietitian recommended, because no one told the provider, and kept losing weight, dropping from about 136 to 125 pounds. Another resident gained about 19 pounds in a month, but staff did not reweigh them or tell the provider or the dietitian.</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
@@ -8338,8 +8386,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415079/health/health-inspection?date=2024-03-15</t>
         </is>
       </c>
-      <c r="H178" s="4" t="inlineStr"/>
-      <c r="I178" s="3" t="inlineStr"/>
+      <c r="H178" s="4" t="inlineStr">
+        <is>
+          <t>A resident with a deep pressure wound at the base of the spine was given no pain medicine before wound care, even though the wound doctor had recommended it. The resident yelled, swore, and complained of pain throughout the treatment, and the nurse kept going until she was done.</t>
+        </is>
+      </c>
+      <c r="I178" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -8377,8 +8433,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415129/health/complaint-inspection?date=2024-03-15</t>
         </is>
       </c>
-      <c r="H179" s="4" t="inlineStr"/>
-      <c r="I179" s="3" t="inlineStr"/>
+      <c r="H179" s="4" t="inlineStr">
+        <is>
+          <t>When a resident with diabetes was found unresponsive with a blood sugar of 31, a nurse injected only the sterile water from the emergency glucagon kit without mixing in the medicine, because she had never been trained to use it. Another nurse noticed and gave a proper second dose before the resident was taken to the hospital, and five other nurses also had no record of glucagon training.</t>
+        </is>
+      </c>
+      <c r="I179" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
@@ -8416,8 +8480,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415129/health/complaint-inspection?date=2024-03-15</t>
         </is>
       </c>
-      <c r="H180" s="4" t="inlineStr"/>
-      <c r="I180" s="3" t="inlineStr"/>
+      <c r="H180" s="4" t="inlineStr">
+        <is>
+          <t>Nurses gave a resident with diabetes insulin several times when the order said to hold it because the blood sugar was below 200, and one nurse said she could not see the full order on the screen. After a 40-unit dose, the resident was found unresponsive and sweaty with a blood sugar of 31, needed emergency treatment, and was admitted to the hospital confused.</t>
+        </is>
+      </c>
+      <c r="I180" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -8455,8 +8527,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415129/health/complaint-inspection?date=2024-03-11</t>
         </is>
       </c>
-      <c r="H181" s="4" t="inlineStr"/>
-      <c r="I181" s="3" t="inlineStr"/>
+      <c r="H181" s="4" t="inlineStr">
+        <is>
+          <t>A resident was sent home with another resident's medicines, including a water pill, a nerve pain drug, an antibiotic, a thyroid drug, and a diabetes drug, and no one reviewed the medicines or instructions with the family. The resident took them for 5 days, and the family said the resident became confused and fell twice before a doctor caught the mistake.</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
@@ -8494,8 +8574,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415032/health/complaint-inspection?date=2024-03-01</t>
         </is>
       </c>
-      <c r="H182" s="4" t="inlineStr"/>
-      <c r="I182" s="3" t="inlineStr"/>
+      <c r="H182" s="4" t="inlineStr">
+        <is>
+          <t>A resident over 100 years old with severe dementia was found partly out of bed with their legs against a hot electric radiator, and had painful, blistered burns on both knees and the right ankle that were treated with morphine. Radiators throughout the building measured 133 to 153 degrees Fahrenheit, and the facility had no safety measures to keep residents from being burned by them.</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -8533,8 +8621,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/complaint-inspection?date=2024-03-01</t>
         </is>
       </c>
-      <c r="H183" s="4" t="inlineStr"/>
-      <c r="I183" s="3" t="inlineStr"/>
+      <c r="H183" s="4" t="inlineStr">
+        <is>
+          <t>A resident with kidney disease, diabetes, and cancer was sent home with a bag of another resident's medicines, including a blood thinner, a diabetes drug, and a water pill, after a nurse grabbed the wrong bag without checking. The family got no teaching about the medicines and found the mistake at home, and two other residents' records had no discharge summary.</t>
+        </is>
+      </c>
+      <c r="I183" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
@@ -8572,8 +8668,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/complaint-inspection?date=2024-02-27</t>
         </is>
       </c>
-      <c r="H184" s="4" t="inlineStr"/>
-      <c r="I184" s="3" t="inlineStr"/>
+      <c r="H184" s="4" t="inlineStr">
+        <is>
+          <t>A legally blind resident who had refused to give up the private room they had lived in for 5 years came back from the hospital to find their belongings boxed up and moved to a shared room without their permission. The resident tripped over the boxes and fell, became very upset, and was admitted to a hospital psychiatric unit.</t>
+        </is>
+      </c>
+      <c r="I184" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -8611,8 +8715,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/complaint-inspection?date=2024-02-15</t>
         </is>
       </c>
-      <c r="H185" s="4" t="inlineStr"/>
-      <c r="I185" s="3" t="inlineStr"/>
+      <c r="H185" s="4" t="inlineStr">
+        <is>
+          <t>A resident with diabetes who was normally alert was found on the floor in the middle of the night confused, but the nurse did not check the resident's blood sugar and did not contact a doctor until hours later. In the morning the resident was barely responding with a blood sugar of 57, needed an emergency injection, and was sent to the hospital.</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
@@ -8650,8 +8762,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415050/health/health-inspection?date=2024-01-22</t>
         </is>
       </c>
-      <c r="H186" s="4" t="inlineStr"/>
-      <c r="I186" s="3" t="inlineStr"/>
+      <c r="H186" s="4" t="inlineStr">
+        <is>
+          <t>Nurses cleaned blood sugar meters shared by several residents with alcohol pads instead of the disinfectant wipes the maker requires to prevent spreading infections carried in blood. One of the residents tested with a shared meter had hepatitis B, a virus spread through blood, and one nurse said he did not have the right wipes on his cart.</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -8689,8 +8809,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415087/health/complaint-inspection?date=2024-01-17</t>
         </is>
       </c>
-      <c r="H187" s="4" t="inlineStr"/>
-      <c r="I187" s="3" t="inlineStr"/>
+      <c r="H187" s="4" t="inlineStr">
+        <is>
+          <t>After a resident's foot got caught under a wheelchair a nurse was pushing and the resident fell, the nurse did not check for injuries or tell a provider and sent the resident on to dialysis. Staff there found a large swollen bruise on the left thigh and a left leg shorter than the right, and the resident was hospitalized with a broken thigh bone.</t>
+        </is>
+      </c>
+      <c r="I187" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
@@ -8728,8 +8856,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415087/health/complaint-inspection?date=2024-01-17</t>
         </is>
       </c>
-      <c r="H188" s="4" t="inlineStr"/>
-      <c r="I188" s="3" t="inlineStr"/>
+      <c r="H188" s="4" t="inlineStr">
+        <is>
+          <t>A nurse pushed a resident with dementia in a wheelchair that had no footrests, and the resident's leg got caught under the wheel and the resident fell to the floor. The resident was hospitalized with a badly broken left thigh bone near an old knee replacement, and the hospital's bone specialists recommended amputating the leg above the knee.</t>
+        </is>
+      </c>
+      <c r="I188" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
@@ -8767,8 +8903,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415106/health/health-inspection?date=2024-01-12</t>
         </is>
       </c>
-      <c r="H189" s="4" t="inlineStr"/>
-      <c r="I189" s="3" t="inlineStr"/>
+      <c r="H189" s="4" t="inlineStr">
+        <is>
+          <t>A resident who weighed about 250 pounds and needed two staff to turn was left with one nursing assistant during a bath on a shower stretcher, and fell off it when, the resident said, a side rail broke. The resident was found face down in a pool of blood with a forehead cut that needed 11 stitches and a swollen, bruised eye, and the facility did not investigate the fall.</t>
+        </is>
+      </c>
+      <c r="I189" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
@@ -8806,8 +8950,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415067/health/health-inspection?date=2024-01-05</t>
         </is>
       </c>
-      <c r="H190" s="4" t="inlineStr"/>
-      <c r="I190" s="3" t="inlineStr"/>
+      <c r="H190" s="4" t="inlineStr">
+        <is>
+          <t>A resident recovering from a leg amputation drank very little for days, had repeated diarrhea, and had blood tests showing dehydration, but staff did not track urine output, and the resident got IV fluids only the evening before dying at the facility. Other residents also drank far less than they needed or kept losing weight without a recommended supplement being started or the provider being told.</t>
+        </is>
+      </c>
+      <c r="I190" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
@@ -8845,8 +8997,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415067/health/health-inspection?date=2024-01-05</t>
         </is>
       </c>
-      <c r="H191" s="4" t="inlineStr"/>
-      <c r="I191" s="3" t="inlineStr"/>
+      <c r="H191" s="4" t="inlineStr">
+        <is>
+          <t>Nurses kept giving a resident a water pill after it was ordered held because blood tests showed dehydration, did not give the ordered diarrhea medicine, and did not track urine output. The resident grew lethargic and confused, staff told the worried family the resident was not getting the wrong medicines, and the resident died at the facility the morning after finally getting IV fluids.</t>
+        </is>
+      </c>
+      <c r="I191" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
@@ -8884,8 +9044,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415067/health/health-inspection?date=2024-01-05</t>
         </is>
       </c>
-      <c r="H192" s="4" t="inlineStr"/>
-      <c r="I192" s="3" t="inlineStr"/>
+      <c r="H192" s="4" t="inlineStr">
+        <is>
+          <t>A resident whose blood tests showed dehydration was given a water pill (torsemide) four more times after the provider ordered it held, including a double dose, and was never given the ordered diarrhea medicine on five days with diarrhea. The resident, who was dehydrated, died at the facility.</t>
+        </is>
+      </c>
+      <c r="I192" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
@@ -8923,8 +9091,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415031/health/complaint-inspection?date=2023-12-28</t>
         </is>
       </c>
-      <c r="H193" s="4" t="inlineStr"/>
-      <c r="I193" s="3" t="inlineStr"/>
+      <c r="H193" s="4" t="inlineStr">
+        <is>
+          <t>A resident with heart failure gained weight and had swelling that no one acted on, and nursing assistants who saw the resident short of breath and in distress did not tell a nurse. An inspector found the resident breathing heavily with a blood oxygen level of 65 percent, and the resident was rushed to the hospital and admitted with respiratory failure caused by heart failure.</t>
+        </is>
+      </c>
+      <c r="I193" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
@@ -8962,8 +9138,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415031/health/complaint-inspection?date=2023-12-28</t>
         </is>
       </c>
-      <c r="H194" s="4" t="inlineStr"/>
-      <c r="I194" s="3" t="inlineStr"/>
+      <c r="H194" s="4" t="inlineStr">
+        <is>
+          <t>A new deep pressure sore found on a resident's tailbone went untreated for 5 days because the wound doctor's recommended treatment was never started. In that time the wound got worse, growing from 1.5 to 2.8 centimeters long.</t>
+        </is>
+      </c>
+      <c r="I194" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Harm citation summaries: batch 5 (19 citations)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PVPrLRkDuJ4YCTTu2Vxqj5
</commit_message>
<xml_diff>
--- a/pipeline/harm_summaries.xlsx
+++ b/pipeline/harm_summaries.xlsx
@@ -9185,8 +9185,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415078/health/complaint-inspection?date=2023-12-26</t>
         </is>
       </c>
-      <c r="H195" s="4" t="inlineStr"/>
-      <c r="I195" s="3" t="inlineStr"/>
+      <c r="H195" s="4" t="inlineStr">
+        <is>
+          <t>A nurse gave a resident with a breathing tube in the neck three seizure drugs, including the strong sedative phenobarbital, and an injection of the blood thinner Lovenox that were all meant for the resident next door, without checking who the resident was. This resident had earlier been taken off Lovenox because it made them cough up blood, and follow-up blood work the doctor ordered was not done.</t>
+        </is>
+      </c>
+      <c r="I195" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
@@ -9224,8 +9232,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415079/health/complaint-inspection?date=2023-12-26</t>
         </is>
       </c>
-      <c r="H196" s="4" t="inlineStr"/>
-      <c r="I196" s="3" t="inlineStr"/>
+      <c r="H196" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe dementia who was known to wander and had gotten out before left a locked unit and walked out the front door past the receptionist, who did not recognize the resident under layers of clothes. The resident was found a few streets away on a day when temperatures were between 21 and 36 degrees Fahrenheit.</t>
+        </is>
+      </c>
+      <c r="I196" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
@@ -9263,8 +9279,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415023/health/complaint-inspection?date=2023-12-13</t>
         </is>
       </c>
-      <c r="H197" s="4" t="inlineStr"/>
-      <c r="I197" s="3" t="inlineStr"/>
+      <c r="H197" s="4" t="inlineStr">
+        <is>
+          <t>During an outbreak of RSV (a contagious respiratory virus), sick residents were on the wrong precautions, staff went into their rooms without the needed gowns, gloves, and eye protection, and a newly coughing resident was not isolated. Several residents had dangerously low oxygen levels, two were hospitalized with septic shock and RSV, and one of them died.</t>
+        </is>
+      </c>
+      <c r="I197" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="3" t="inlineStr">
@@ -9302,8 +9326,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415044/health/complaint-inspection?date=2023-12-11</t>
         </is>
       </c>
-      <c r="H198" s="4" t="inlineStr"/>
-      <c r="I198" s="3" t="inlineStr"/>
+      <c r="H198" s="4" t="inlineStr">
+        <is>
+          <t>A resident recovering from spine surgery who needed a back brace, a gait belt, and two staff for every transfer was moved alone by an unlicensed nursing assistant without the brace or the belt, and fell. Emergency responders had to help get the resident off the floor, and afterward the resident had more pain, needed pain medicine and a standing aid for transfers, and was more afraid of falling.</t>
+        </is>
+      </c>
+      <c r="I198" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
@@ -9341,8 +9373,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415044/health/complaint-inspection?date=2023-12-11</t>
         </is>
       </c>
-      <c r="H199" s="4" t="inlineStr"/>
-      <c r="I199" s="3" t="inlineStr"/>
+      <c r="H199" s="4" t="inlineStr">
+        <is>
+          <t>The facility let new nursing assistants who had not yet received their state licenses work on their own with residents, a practice the administrator said went back 30 years. One of them moved a resident recovering from spine surgery alone and without the required back brace, and the resident fell and had more pain.</t>
+        </is>
+      </c>
+      <c r="I199" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
@@ -9380,8 +9420,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/complaint-inspection?date=2023-12-07</t>
         </is>
       </c>
-      <c r="H200" s="4" t="inlineStr"/>
-      <c r="I200" s="3" t="inlineStr"/>
+      <c r="H200" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe dementia was sexually assaulted in bed by their roommate, who also has dementia, and was trying to push the roommate away and yelling stop when staff found them. The roommate had repeatedly tried to get into the resident's bed and other residents' beds before, and police were not called after the assault.</t>
+        </is>
+      </c>
+      <c r="I200" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
@@ -9419,8 +9467,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415099/health/complaint-inspection?date=2023-12-07</t>
         </is>
       </c>
-      <c r="H201" s="4" t="inlineStr"/>
-      <c r="I201" s="3" t="inlineStr"/>
+      <c r="H201" s="4" t="inlineStr">
+        <is>
+          <t>A resident with Alzheimer's disease on hospice repeatedly wandered at night, tried to get into a roommate's and other residents' beds, and became combative, but the behavior care plan was never reviewed or updated to address it. The resident later sexually assaulted the roommate, who also has dementia.</t>
+        </is>
+      </c>
+      <c r="I201" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="3" t="inlineStr">
@@ -9458,8 +9514,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415091/health/health-inspection?date=2023-11-30</t>
         </is>
       </c>
-      <c r="H202" s="4" t="inlineStr"/>
-      <c r="I202" s="3" t="inlineStr"/>
+      <c r="H202" s="4" t="inlineStr">
+        <is>
+          <t>Nurses had not been trained to use a heated hot pack machine and left a resident with one-sided paralysis, who cannot reposition on their own, lying on a hot pack wrapped in too few towels without watching. The resident got a burn on the lower back that needed burn cream.</t>
+        </is>
+      </c>
+      <c r="I202" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -9497,8 +9561,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415038/health/complaint-inspection?date=2023-11-22</t>
         </is>
       </c>
-      <c r="H203" s="4" t="inlineStr"/>
-      <c r="I203" s="3" t="inlineStr"/>
+      <c r="H203" s="4" t="inlineStr">
+        <is>
+          <t>A newly admitted resident never got their daily methadone or their anxiety medicine (Klonopin), because the methadone order was faxed to the wrong clinic and the Klonopin prescription never reached the pharmacy. The resident became agitated, screamed, and threw things, and was taken to the hospital with body aches and concerns about methadone withdrawal.</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="3" t="inlineStr">
@@ -9536,8 +9608,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415008/health/complaint-inspection?date=2023-11-21</t>
         </is>
       </c>
-      <c r="H204" s="4" t="inlineStr"/>
-      <c r="I204" s="3" t="inlineStr"/>
+      <c r="H204" s="4" t="inlineStr">
+        <is>
+          <t>A resident with no history of seizures had seizure activity and high blood pressure, but the nurse did not tell the doctor, who said she would have sent the resident to the hospital. The resident later stopped breathing and had no pulse, needed CPR, and was admitted to the hospital with sepsis and a severe bowel infection.</t>
+        </is>
+      </c>
+      <c r="I204" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
@@ -9575,8 +9655,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415120/health/complaint-inspection?date=2023-11-17</t>
         </is>
       </c>
-      <c r="H205" s="4" t="inlineStr"/>
-      <c r="I205" s="3" t="inlineStr"/>
+      <c r="H205" s="4" t="inlineStr">
+        <is>
+          <t>A coworker saw an agency nursing assistant hit a resident with severe memory problems in the face with pillows and stretch another resident's legs so hard the resident screamed in pain. The same aide woke a third resident by slamming silverware down and laughed, which frightened that resident, and the nurse who was told did not remove the aide or report it right away.</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="3" t="inlineStr">
@@ -9614,8 +9702,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415084/health/complaint-inspection?date=2023-11-14</t>
         </is>
       </c>
-      <c r="H206" s="4" t="inlineStr"/>
-      <c r="I206" s="3" t="inlineStr"/>
+      <c r="H206" s="4" t="inlineStr">
+        <is>
+          <t>A nurse gave a resident on hospice, who has liver and lung disease, a 60 mg dose of methadone that was meant for the roommate. The resident was found on the floor with pinpoint pupils, slowed breathing, and low oxygen, needed two doses of Narcan to reverse the overdose, and was admitted to a hospital critical care unit.</t>
+        </is>
+      </c>
+      <c r="I206" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -9653,8 +9749,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415098/health/health-inspection?date=2023-11-10</t>
         </is>
       </c>
-      <c r="H207" s="4" t="inlineStr"/>
-      <c r="I207" s="3" t="inlineStr"/>
+      <c r="H207" s="4" t="inlineStr">
+        <is>
+          <t>A nurse used one shared blood sugar meter on three residents, one of them with hepatitis C, without properly disinfecting it between them, pulled out bloody test strips by hand, and let the dirty meter touch clean supplies. A resident with MRSA (a drug-resistant infection) was also taken off contact precautions without the required follow-up tests, putting residents at risk of infection.</t>
+        </is>
+      </c>
+      <c r="I207" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="3" t="inlineStr">
@@ -9692,8 +9796,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415064/health/complaint-inspection?date=2023-11-06</t>
         </is>
       </c>
-      <c r="H208" s="4" t="inlineStr"/>
-      <c r="I208" s="3" t="inlineStr"/>
+      <c r="H208" s="4" t="inlineStr">
+        <is>
+          <t>The facility admitted a resident who was a high-risk registered sex offender without checking, which its own rules forbid, and put no protections in place for other residents after learning about it. Weeks later, after this resident had also smacked a nurse on the buttocks, staff saw the resident touch a resident with severe dementia on the thighs and breasts.</t>
+        </is>
+      </c>
+      <c r="I208" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
@@ -9731,8 +9843,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415064/health/complaint-inspection?date=2023-11-06</t>
         </is>
       </c>
-      <c r="H209" s="4" t="inlineStr"/>
-      <c r="I209" s="3" t="inlineStr"/>
+      <c r="H209" s="4" t="inlineStr">
+        <is>
+          <t>Staff were not told to closely supervise a resident known to be a high-risk registered sex offender, who went into and sat outside the rooms of residents with severe dementia. The resident touched a resident with severe dementia on the thighs and breasts in the dining room.</t>
+        </is>
+      </c>
+      <c r="I209" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="3" t="inlineStr">
@@ -9770,8 +9890,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415044/health/health-inspection?date=2023-10-30</t>
         </is>
       </c>
-      <c r="H210" s="4" t="inlineStr"/>
-      <c r="I210" s="3" t="inlineStr"/>
+      <c r="H210" s="4" t="inlineStr">
+        <is>
+          <t>A resident was yellow (jaundiced) for about two weeks and had stomach pain, but staff did not tell the doctor, kept giving daily Tylenol that a specialist said to avoid, and never passed on an ultrasound result recommending a CT scan. The resident was found unresponsive and admitted to intensive care with a gallstone blocking the bile duct and severe anemia that needed 5 units of blood.</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
@@ -9809,8 +9937,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415044/health/health-inspection?date=2023-10-30</t>
         </is>
       </c>
-      <c r="H211" s="4" t="inlineStr"/>
-      <c r="I211" s="3" t="inlineStr"/>
+      <c r="H211" s="4" t="inlineStr">
+        <is>
+          <t>A resident had burning when urinating, dark urine, and lower belly or side pain, but staff did not tell the provider or test the urine for 13 days, until an inspector raised it. The test then showed a urinary tract infection, and the resident still had burning while on antibiotics.</t>
+        </is>
+      </c>
+      <c r="I211" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="3" t="inlineStr">
@@ -9848,8 +9984,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415085/health/health-inspection?date=2023-10-25</t>
         </is>
       </c>
-      <c r="H212" s="4" t="inlineStr"/>
-      <c r="I212" s="3" t="inlineStr"/>
+      <c r="H212" s="4" t="inlineStr">
+        <is>
+          <t>A resident with Alzheimer's disease and a history of past abuse, whose care plan called for two staff, a stuffed comfort dog, and stepping away when the resident got upset, was cleaned by one aide who did not know the plan. The resident lay naked yelling "Help me!" and pushing the aide's hand away while care went on, and staff said this distress happened often.</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
@@ -9887,8 +10031,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415029/health/health-inspection?date=2023-10-13</t>
         </is>
       </c>
-      <c r="H213" s="4" t="inlineStr"/>
-      <c r="I213" s="3" t="inlineStr"/>
+      <c r="H213" s="4" t="inlineStr">
+        <is>
+          <t>A resident with schizophrenia and other mental health conditions was kept under a behavior contract that took away coffee and activities as punishment and threatened a move to another facility, which neither the resident's psychiatric doctor nor regular doctor agreed with. The resident's coffee-seeking and aggressive behavior grew worse.</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Harm citation summaries: batch 6 (10 citations)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PVPrLRkDuJ4YCTTu2Vxqj5
</commit_message>
<xml_diff>
--- a/pipeline/harm_summaries.xlsx
+++ b/pipeline/harm_summaries.xlsx
@@ -10078,8 +10078,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415057/health/health-inspection?date=2023-09-22</t>
         </is>
       </c>
-      <c r="H214" s="4" t="inlineStr"/>
-      <c r="I214" s="3" t="inlineStr"/>
+      <c r="H214" s="4" t="inlineStr">
+        <is>
+          <t>A resident who had hallucinations from the antibiotic Invanz in February was given it again in September because the reaction was never added to their allergy list, and again had frightening hallucinations and confusion. The same resident never had an ordered urology visit, and a hospice nurse's recommendation to restart anxiety medicine for another resident was never acted on.</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
@@ -10117,8 +10125,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415057/health/health-inspection?date=2023-09-22</t>
         </is>
       </c>
-      <c r="H215" s="4" t="inlineStr"/>
-      <c r="I215" s="3" t="inlineStr"/>
+      <c r="H215" s="4" t="inlineStr">
+        <is>
+          <t>A resident with deep pressure wounds and a bone infection refused a dressing change because of pain, and staff did not ask a provider for pain medicine sooner than every 12 hours and told the resident to write their concerns down for the doctor's next visit. Another resident's new severe back and leg pain was not reported to the doctor for 4 days.</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="3" t="inlineStr">
@@ -10156,8 +10172,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415057/health/health-inspection?date=2023-09-22</t>
         </is>
       </c>
-      <c r="H216" s="4" t="inlineStr"/>
-      <c r="I216" s="3" t="inlineStr"/>
+      <c r="H216" s="4" t="inlineStr">
+        <is>
+          <t>A resident was given the antibiotic Invanz again even though it had caused hallucinations months earlier, because the reaction was never recorded as an allergy. The resident again had hallucinations and confusion, and a nurse said the resident seemed to be in severe mental distress.</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
@@ -10195,8 +10219,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/health-inspection?date=2023-07-06</t>
         </is>
       </c>
-      <c r="H217" s="4" t="inlineStr"/>
-      <c r="I217" s="3" t="inlineStr"/>
+      <c r="H217" s="4" t="inlineStr">
+        <is>
+          <t>A nurse, with no doctor's order, marked a hospice resident with brain cancer as allowed nothing by mouth and stopped the resident's steroid medicine for brain swelling. The resident got no food or drink for 6 days before dying, and staff also skipped ordered blood sugar rechecks and did not follow wound care orders for another resident.</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="3" t="inlineStr">
@@ -10234,8 +10266,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/health-inspection?date=2023-07-06</t>
         </is>
       </c>
-      <c r="H218" s="4" t="inlineStr"/>
-      <c r="I218" s="3" t="inlineStr"/>
+      <c r="H218" s="4" t="inlineStr">
+        <is>
+          <t>A hospice resident with brain cancer who had been eating was made nothing by mouth by a nurse with no doctor's order, which hospice, the dietitian, and the doctor said they would never recommend. The resident got no food or fluids and showed signs of dehydration in the 6 days before dying, and other residents' wound treatments did not match the wound doctor's recommendations.</t>
+        </is>
+      </c>
+      <c r="I218" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
@@ -10273,8 +10313,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/health-inspection?date=2023-07-06</t>
         </is>
       </c>
-      <c r="H219" s="4" t="inlineStr"/>
-      <c r="I219" s="3" t="inlineStr"/>
+      <c r="H219" s="4" t="inlineStr">
+        <is>
+          <t>A resident with brain cancer on hospice was given no fluids for 6 days because a nurse entered a nothing-by-mouth order without a doctor's approval. The resident's urine dropped and darkened, a sign of dehydration, and the resident died on the sixth day.</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="3" t="inlineStr">
@@ -10312,8 +10360,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415059/health/health-inspection?date=2023-07-06</t>
         </is>
       </c>
-      <c r="H220" s="4" t="inlineStr"/>
-      <c r="I220" s="3" t="inlineStr"/>
+      <c r="H220" s="4" t="inlineStr">
+        <is>
+          <t>A doctor signed a batch of orders without reading them, which approved a nurse's unauthorized order that a hospice resident with brain cancer get nothing by mouth. Because no doctor caught the error, the resident went without food, fluids, and a steroid for brain swelling in the 6 days before dying.</t>
+        </is>
+      </c>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
@@ -10351,8 +10407,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415119/health/health-inspection?date=2023-06-08</t>
         </is>
       </c>
-      <c r="H221" s="4" t="inlineStr"/>
-      <c r="I221" s="3" t="inlineStr"/>
+      <c r="H221" s="4" t="inlineStr">
+        <is>
+          <t>A resident with severe malnutrition lost about 34 pounds in under two months, and the ice cream ordered with every meal to help never came because the order never reached the kitchen. Another resident with severe malnutrition lost 7.5 pounds without being reweighed or getting any new help.</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="3" t="inlineStr">
@@ -10390,8 +10454,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415119/health/health-inspection?date=2023-06-08</t>
         </is>
       </c>
-      <c r="H222" s="4" t="inlineStr"/>
-      <c r="I222" s="3" t="inlineStr"/>
+      <c r="H222" s="4" t="inlineStr">
+        <is>
+          <t>A resident with a severe nerve pain condition in both legs often rated their pain 10 out of 10, but no new pain treatment was started after a neurologist recommended options, because the doctor said he was not licensed to prescribe them.</t>
+        </is>
+      </c>
+      <c r="I222" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
@@ -10429,8 +10501,16 @@
           <t>https://www.medicare.gov/care-compare/inspections/pdf/nursing-home/415061/health/health-inspection?date=2023-05-22</t>
         </is>
       </c>
-      <c r="H223" s="4" t="inlineStr"/>
-      <c r="I223" s="3" t="inlineStr"/>
+      <c r="H223" s="4" t="inlineStr">
+        <is>
+          <t>Staff did not catch severe weight loss in several residents. One resident with dementia lost about 25 pounds, nearly 20 percent of their weight, in about a month, because weekly weights were skipped and no one told the provider, family, or dietitian. Another lost over 7 percent of their weight in 3 weeks, and a third went about 4 weeks without an ordered protein supplement while their protein levels dropped.</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>Claude (draft for kg's review)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I223"/>

</xml_diff>